<commit_message>
Registro compensi v1.1: riferimenti normativi 2027
</commit_message>
<xml_diff>
--- a/download/registro-compensi-occasionali.xlsx
+++ b/download/registro-compensi-occasionali.xlsx
@@ -648,7 +648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:A36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="115" customWidth="1" min="1" max="1"/>
@@ -795,43 +795,88 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>• Ritenuta 20% su compensi di lavoro autonomo anche non abituale: art. 25, primo comma, DPR 600/1973 (normattiva.it). Dal 1/1/2027 la materia passa al</t>
+          <t>• Ritenuta 20% su compensi di lavoro autonomo anche non abituale: art. 25, primo comma, DPR 600/1973 (normattiva.it).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  D.Lgs. 33/2025 (Testo unico versamenti e riscossione; decorrenza fissata dal DL 200/2025): l'aliquota va riverificata a gennaio 2027.</t>
+          <t>• Imposta di bollo 2,00 € su ricevute oltre 77,47 €: DPR 642/1972, Tariffa allegato A, parte I, art. 13 e nota 2; Agenzia delle Entrate, risposta a interpello 129/2024.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>• Imposta di bollo 2,00 € su ricevute oltre 77,47 €: DPR 642/1972, Tariffa allegato A, parte I, art. 13 e nota 2; Agenzia delle Entrate, risposta a interpello 129/2024.</t>
+          <t>• Soglia 5.000 € e Gestione separata INPS: art. 44, comma 2, DL 269/2003 (normattiva.it).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>• Soglia 5.000 € e Gestione separata INPS: art. 44, comma 2, DL 269/2003 (normattiva.it).</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
           <t>• Reddito di lavoro autonomo occasionale al netto delle spese specificamente inerenti: art. 67, comma 1, lett. l) e art. 71, comma 2, DPR 917/1986 (TUIR).</t>
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr"/>
+    </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr"/>
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>DAL 1° GENNAIO 2027 CAMBIANO I NUMERI DEGLI ARTICOLI (testi letti in Gazzetta Ufficiale e su Normattiva il 31/10/2026)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>• Ritenuta 20%: art. 38, comma 1, D.Lgs. 33/2025 (Testo unico versamenti e riscossione), al posto dell'art. 25 DPR 600/1973. Decorrenza: art. 243, data 1/1/2027 (DL 200/2025).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>• Compenso occasionale come reddito diverso: art. 76, comma 1, lett. t), D.Lgs. 117/2026 (nuovo TUIR), al posto dell'art. 67, comma 1, lett. l), DPR 917/1986. Decorrenza: art. 377.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>• IVA, requisito di abitualita': art. 4, comma 1, D.Lgs. 10/2026 (Testo unico IVA), al posto dell'art. 5 DPR 633/1972. Decorrenza: art. 171.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>• Nei testi letti l'aliquota della ritenuta resta il 20%: le formule di questo foglio non cambiano.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>• Da verificare: il nuovo riferimento per il bollo e quello per le spese inerenti (oggi art. 71, comma 2, TUIR). Soglia INPS (DL 269/2003): norma non compresa nei tre testi unici.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>• Tabella completa e aggiornamenti: https://lumen-ledger.github.io/it/riferimenti-normativi-2027-ricevute/</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>Questo foglio e' informazione generale e strumento di calcolo, non consulenza fiscale o legale. Verifica il tuo caso con un professionista o un CAF.</t>
         </is>
@@ -14383,7 +14428,7 @@
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
-          <t>art. 25 DPR 600/1973 (dal 2027: D.Lgs. 33/2025) — verificato 31/10/2026</t>
+          <t>art. 25 DPR 600/1973; dal 1/1/2027 art. 38, c. 1, D.Lgs. 33/2025 (20%) — verificato 31/10/2026</t>
         </is>
       </c>
     </row>
@@ -14398,7 +14443,7 @@
       </c>
       <c r="C3" s="11" t="inlineStr">
         <is>
-          <t>DPR 642/1972, Tariffa all. A, parte I, art. 13</t>
+          <t>DPR 642/1972, Tariffa all. A, parte I, art. 13 (riferimento dal 2027 da verificare)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Spese inerenti 2027 (art. 80 c.2 D.Lgs. 117/2026), registro compensi v1.2
</commit_message>
<xml_diff>
--- a/download/registro-compensi-occasionali.xlsx
+++ b/download/registro-compensi-occasionali.xlsx
@@ -648,7 +648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A36"/>
+  <dimension ref="A1:A37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="115" customWidth="1" min="1" max="1"/>
@@ -854,29 +854,36 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>• Nei testi letti l'aliquota della ritenuta resta il 20%: le formule di questo foglio non cambiano.</t>
+          <t>• Spese specificamente inerenti (reddito = incassi meno spese): art. 80, comma 2, D.Lgs. 117/2026, al posto dell'art. 71, comma 2, DPR 917/1986. Stesso testo.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>• Da verificare: il nuovo riferimento per il bollo e quello per le spese inerenti (oggi art. 71, comma 2, TUIR). Soglia INPS (DL 269/2003): norma non compresa nei tre testi unici.</t>
+          <t>• Nei testi letti l'aliquota della ritenuta resta il 20%: le formule di questo foglio non cambiano.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
+          <t>• Bollo: D.Lgs. 123/2025, allegato 3, Tariffa parte I (numero dell'articolo da verificare). Soglia INPS (DL 269/2003): norma non compresa nei tre testi unici.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
           <t>• Tabella completa e aggiornamenti: https://lumen-ledger.github.io/it/riferimenti-normativi-2027-ricevute/</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr"/>
-    </row>
     <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+      <c r="A36" s="3" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>Questo foglio e' informazione generale e strumento di calcolo, non consulenza fiscale o legale. Verifica il tuo caso con un professionista o un CAF.</t>
         </is>

</xml_diff>